<commit_message>
Realistic sample set: six invoice layouts, scan simulation, OCR fallback, instalment and combined payments
- sample_gen/: 12 invented vendors with fixed regional conventions, six
  Jinja2/Chromium templates (UK service, US letter, freelancer, e-invoice
  grid, statement, thermal receipt), flatbed and phone-photo scan simulation
  producing image-only PDFs. generate_sample_data.py plants nine fault kinds
  and writes EXPECTED.json ground truth plus a 32-file browser subset.
- extract.py: EU/US/plain number formats, six date formats with day/month
  disambiguation, more total labels, OCR fallback (pymupdf + tesseract,
  raw pass first, deskew/despeckle rescue), extraction_method on Invoice.
- match.py: paid_in_instalments and combined_payment recognised instead of
  reported as mismatches; coverage check counts instalment rows.
- report.py: Read Via column.
- tests: ground-truth scorer, clean set must read 100%, OCR floors opt-in.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/ledger.xlsx
+++ b/sample_data/ledger.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,9 +48,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,128 +444,113 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>45667</v>
+        <v>45669</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Payment to Nordway Logistics</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>INV-1001</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>858.34</v>
+          <t>WRENFIELD SOFTWARE LTD WS-0622</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>741.98</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>45671</v>
+        <v>45677</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Payment to Cedar &amp; Finch Consulting</t>
+          <t>Saltmarsh Coffee Roasters - invoice 478</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>INV-1002</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>463.94</v>
+          <t>478</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>339.32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>45675</v>
+        <v>45677</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Payment to Pinehollow Office Co</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>INV-1003</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1604.13</v>
+          <t>Cedar &amp; Finch Consulting - invoice CF-2025-507</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>818.85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>45683</v>
+        <v>45679</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Payment to Amberlake Facilities</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>INV-1005</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1341.81</v>
+          <t>Payment to Meridian Print Services</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>8141.11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>45687</v>
+        <v>45679</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Payment to Bluefern Supplies Ltd</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>INV-1006</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>953.77</v>
+          <t>Wire transfer 160</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>3846.39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>45691</v>
+        <v>45685</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Payment to Nordway Logistics</t>
+          <t>NORDWAY LOGISTICS NW-258</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>INV-1007</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>252.24</v>
+          <t>NW-258</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>5374.15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>45693</v>
+        <v>45686</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Wire transfer - Amberlake Facilities</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>875</v>
+          <t>Wire transfer BF-00434</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BF-00434</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>2413.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>45695</v>
+        <v>45690</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -573,155 +559,1478 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>INV-1008</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1326.95</v>
+          <t>CF-2025-509</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>2469.34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>45699</v>
+        <v>45690</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Payment to Pinehollow Office Co</t>
+          <t>Karadut Yazılım A.Ş. - invoice KDY2025000000198</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>INV-1009</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>205.49</v>
+          <t>KDY2025000000198</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>207617.33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>45703</v>
+        <v>45691</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Payment to Meridian Print Services</t>
+          <t>Payment to Bluefern Supplies Ltd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>INV-1010</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1108.71</v>
+          <t>BF-00436</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1349.38</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>45707</v>
+        <v>45691</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Payment to Amberlake Facilities</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>INV-1011</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>279.27</v>
+          <t>Direct debit  Meridian Print Services</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>312.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>45711</v>
+        <v>45692</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Payment to Bluefern Supplies Ltd</t>
+          <t>Pinehollow Office Co - invoice PH/2025/0768</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>INV-1012</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>326.83</v>
+          <t>PH/2025/0768</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>734.78</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>45715</v>
+        <v>45694</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Payment to Nordway Logistics</t>
+          <t>Payment to Bluefern Supplies Ltd</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>INV-1013</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>1087.9</v>
+          <t>BF-00432</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>661.51</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>45719</v>
+        <v>45694</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Payment to Cedar &amp; Finch Consulting</t>
+          <t>Payment to Nordway Logistics</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>INV-1014</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>2005.22</v>
+          <t>NW-262</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>4105.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>45723</v>
+        <v>45694</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Payment to Pinehollow Office Co</t>
+          <t>BACS Meridian Print Services</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>INV-1015</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>402.27</v>
+          <t>MPS000154</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>3185.87</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>45727</v>
+        <v>45694</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Payment to Meridian Print Services</t>
+          <t>ORRIN BAKKE ELEKTRO AS 164</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>INV-1016</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>628.98</v>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>868.85</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>45697</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Card purchase Orrin Bakke Elektro AS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>166</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>5108.49</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>45698</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NORDWAY LOGISTICS NW-265</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NW-265</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>984.86</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>45699</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Wire transfer 162</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>2992.86</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>45699</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Halden &amp; Roux Avocats - invoice HR-0649</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>HR-0649</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>4649.76</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>45701</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Wire transfer CF-2025-512</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>1834.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>45702</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Wire transfer BF-00434 (balance)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BF-00434</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>2413.8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>45703</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Meridian Print Services - invoice MPS000158</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MPS000158</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>339.55</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>45711</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Saltmarsh Coffee Roasters - invoice 482</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>482</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>110.98</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>45713</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Payment to Halden &amp; Roux Avocats</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>HR-0651</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>1275.9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>45714</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Karadut Yazılım A.Ş. - invoice KDY2025000000203</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KDY2025000000203</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>65649.64999999999</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>45715</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Wire transfer KDY2025000000200</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KDY2025000000200</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>290496.74</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>45719</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Payment to Cedar &amp; Finch Consulting</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CF-2025-513</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>5356.18</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>45719</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Payment to Pinehollow Office Co</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PH/2025/0772</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>2833.65</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>45725</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BACS Nordway Logistics</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>NW-266</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>1457.03</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>45735</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Wire transfer BF-00440</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BF-00440</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>39688.7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>45738</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HALDEN &amp; ROUX AVOCATS HR-0655</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>HR-0655</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>8505.540000000001</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>45742</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Wire transfer CF-2025-517</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CF-2025-517</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>2838.29</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>45743</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Payment to Wrenfield Software Ltd</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>WS-0625</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>2307.2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>45744</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bank charges</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>45745</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Halden &amp; Roux Avocats - invoice HR-0654</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>HR-0654</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>382.2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>45745</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Card purchase Cedar &amp; Finch Consulting</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CF-2025-520</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>3125.95</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>45745</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Wire transfer AF-00176</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AF-00176</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>132615.3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>45747</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Card purchase Pinehollow Office Co</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PH/2025/0774</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>7555.6</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>45747</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Card purchase Tidewell Insurance Brokers</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>1165.75</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BACS Orrin Bakke Elektro AS</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>6718.75</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BACS Karadut Yazılım A.Ş.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>KDY2025000000206</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>133004.16</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>45757</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Payment to Tidewell Insurance Brokers</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>TIB-0000699</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>2330.26</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>45758</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Halden &amp; Roux Avocats - invoice HR-0661</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>HR-0661</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>975.78</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>45761</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Halden &amp; Roux Avocats - invoice HR-0659</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>HR-0659</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>4217.36</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>45765</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Payment to Wrenfield Software Ltd</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>WS-0631</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>3896.98</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>45767</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BACS Saltmarsh Coffee Roasters</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>484</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>596.65</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>45767</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Card purchase Tidewell Insurance Brokers</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TIB-0000702</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>3300.39</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>45768</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Card purchase Karadut Yazılım A.Ş.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>KDY2025000000208</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>259192.27</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>45770</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>BACS Karadut Yazılım A.Ş.</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>78864.08</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>45773</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Card purchase Amberlake Facilities</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>18020.81</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>45774</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>MERIDIAN PRINT SERVICES MPS000161</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>MPS000161</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>182.02</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>45775</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Payment to Wrenfield Software Ltd</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>WS-0629</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>2545.81</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>45777</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Card purchase  Saltmarsh Coffee Roasters</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>46.85</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>45780</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Card purchase Orrin Bakke Elektro AS</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>2305.18</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>45781</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Wire transfer CF-2025-523</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CF-2025-523</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>1557.02</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>45784</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Karadut Yazılım A.Ş. - invoice KDY2025000000212</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>KDY2025000000212</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>88863.38</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>45786</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Wire transfer BF-00439 + WS-0633</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>BF-00439 WS-0633</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>9333.84</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>45788</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Card purchase Bluefern Supplies Ltd</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>BF-00446</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>4136.69</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>45789</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ORRIN BAKKE ELEKTRO AS 174</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>1215.81</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>45790</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Payment to Bluefern Supplies Ltd</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>BF-00442</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>2622.11</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>45790</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Wire transfer AF-00188</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>AF-00188</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>5379.09</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>45791</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Payment to Saltmarsh Coffee Roasters</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>489</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>192.08</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>45792</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SALTMARSH COFFEE ROASTERS 485</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>485</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>202.22</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>45802</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Amberlake Facilities - invoice AF-00184</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>AF-00184</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>10590.53</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>45804</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Card purchase Cedar &amp; Finch Consulting</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>CF-2025-526</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>1599.61</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>45805</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>BACS Wrenfield Software Ltd</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>WS-0636</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>1538.69</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>45805</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>KARADUT YAZILIM A.Ş. KDY2025000000215</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>KDY2025000000215</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>48949.2</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>45805</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Refund Bluefern Supplies Ltd</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>BF-00448</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>-3264.48</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>45806</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Wire transfer MPS000165</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>748.22</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>45808</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Card purchase Amberlake Facilities</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>AF-00190</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>9495.15</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>45810</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Amberlake Facilities - invoice AF-00191</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>AF-00191</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>8839.469999999999</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>45811</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Card purchase Meridian Print Services</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>MPS000168</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>4776.36</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>45813</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>HALDEN &amp; ROUX AVOCATS HR-0666</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>HR-0666</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>1311.34</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>45817</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>BACS Nordway Logistics</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>NW-272</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>1598.16</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>45817</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Amberlake Facilities - invoice AF-00191 (balance)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>AF-00191</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>3788.35</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>45818</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>BACS Halden &amp; Roux Avocats</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>HR-0664</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>6501.48</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>45818</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Payment to Tidewell Insurance Brokers</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TIB-0000705</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>226.53</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>45819</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Wire transfer NW-269</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>NW-269</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>6989.33</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>45820</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Card purchase Cedar &amp; Finch Consulting</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CF-2025-530</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>2347.74</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>45821</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Payment to Wrenfield Software Ltd</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>WS-0640</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>2672.88</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>45823</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>BACS Amberlake Facilities</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>AF-00193</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>15670.64</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>45825</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PINEHOLLOW OFFICE CO PH/2025/0786</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>PH/2025/0786</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>5624.56</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>45827</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BACS Pinehollow Office Co</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>PH/2025/0778</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>1998.52</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>45828</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>BACS Pinehollow Office Co</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>PH/2025/0782</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>10248.93</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>45829</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Card purchase Tidewell Insurance Brokers</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>TIB-0000704</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>830.66</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>45831</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Wire transfer TIB-0000707</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TIB-0000707</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>2250.41</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>45836</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>NORDWAY LOGISTICS NW-274</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>NW-274</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>317.59</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>45837</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Payment to Karadut Yazılım A.Ş.</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>KDY2025000000217</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>126011.64</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Card purchase Wrenfield Software Ltd</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>WS-0641</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>1783.88</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>45846</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Card purchase Nordway Logistics</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>NW-279</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>5167.84</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Orrin Bakke Elektro AS - invoice 178</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>14231.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>